<commit_message>
Eliminate default organism, add taxonomy check
</commit_message>
<xml_diff>
--- a/config/samples.xlsx
+++ b/config/samples.xlsx
@@ -16,17 +16,6 @@
   <calcPr calcMode="auto" iterate="1" iterateCount="100" iterateDelta="0.001"/>
   <webPublishing allowPng="1" css="0" codePage="1252"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="2" count="2">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>Eco72I</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -101,15 +90,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" style="0" width="12.856370192307693"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -138,12 +129,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ref_organism</t>
+          <t>organism</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>organism</t>
+          <t>isolate</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -157,7 +148,7 @@
         </is>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11">
       <c r="A2" t="inlineStr">
         <is>
           <t>4B8</t>
@@ -178,9 +169,14 @@
           <t>4b8</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bdellovibrionota bacterium</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Bdellovibrionota bacterium 4B8</t>
+          <t>KIN4B8</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -188,8 +184,10 @@
           <t>https://www.novoprolabs.com/uploads/vector-maps/pCC1FOS.gb</t>
         </is>
       </c>
-      <c r="J2" t="s">
-        <v>1</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Eco72I</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>